<commit_message>
Correct font glyph sequence; reinstate prior grouping into the replacement glyph. Needs to be reconsidered anyway.
</commit_message>
<xml_diff>
--- a/res/fonts/sortingOrder.xlsx
+++ b/res/fonts/sortingOrder.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacomostert/c43/res/fonts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B747BC-E483-2B44-B015-A613396B4BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{605FAC2C-347D-394F-B466-C1177A483B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="20060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19340" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sortingOrder" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2721" uniqueCount="2025">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2763" uniqueCount="2025">
   <si>
     <t>Code point</t>
   </si>
@@ -6298,7 +6298,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6313,7 +6313,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -6330,7 +6354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6367,6 +6391,18 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -6681,9 +6717,8 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A5,3,4)))</f>
         <v>#</v>
       </c>
-      <c r="H5" s="17" t="str">
-        <f>A5</f>
-        <v>U+0023</v>
+      <c r="H5" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="I5" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H5,3,4)))</f>
@@ -20988,7 +21023,7 @@
       </c>
       <c r="B437" s="5">
         <f>IF(ISNA(VLOOKUP(H437,$A$2:$C$1011,3,1)),C437,VLOOKUP(H437,$A$2:$C$1011,3,1))</f>
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="C437" s="1">
         <v>664</v>
@@ -21007,13 +21042,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A437,3,4)))</f>
         <v>∂</v>
       </c>
-      <c r="H437" s="17" t="str">
-        <f>A437</f>
-        <v>U+2202</v>
+      <c r="H437" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I437" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H437,3,4)))</f>
-        <v>∂</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="438" spans="1:11" s="16" customFormat="1" ht="17" customHeight="1">
@@ -21022,7 +21056,7 @@
       </c>
       <c r="B438" s="5">
         <f>IF(ISNA(VLOOKUP(H438,$A$2:$C$1011,3,1)),C438,VLOOKUP(H438,$A$2:$C$1011,3,1))</f>
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="C438" s="1">
         <v>665</v>
@@ -21041,13 +21075,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A438,3,4)))</f>
         <v>∃</v>
       </c>
-      <c r="H438" s="17" t="str">
-        <f>A438</f>
-        <v>U+2203</v>
+      <c r="H438" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I438" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H438,3,4)))</f>
-        <v>∃</v>
+        <v>Ɐ</v>
       </c>
       <c r="J438" s="4"/>
       <c r="K438" s="2"/>
@@ -21058,7 +21091,7 @@
       </c>
       <c r="B439" s="5">
         <f>IF(ISNA(VLOOKUP(H439,$A$2:$C$1011,3,1)),C439,VLOOKUP(H439,$A$2:$C$1011,3,1))</f>
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="C439" s="1">
         <v>666</v>
@@ -21077,13 +21110,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A439,3,4)))</f>
         <v>∄</v>
       </c>
-      <c r="H439" s="17" t="str">
-        <f>A439</f>
-        <v>U+2204</v>
+      <c r="H439" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I439" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H439,3,4)))</f>
-        <v>∄</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="440" spans="1:11" ht="17" customHeight="1">
@@ -21092,7 +21124,7 @@
       </c>
       <c r="B440" s="5">
         <f>IF(ISNA(VLOOKUP(H440,$A$2:$C$1011,3,1)),C440,VLOOKUP(H440,$A$2:$C$1011,3,1))</f>
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="C440" s="1">
         <v>667</v>
@@ -21111,13 +21143,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A440,3,4)))</f>
         <v>∅</v>
       </c>
-      <c r="H440" s="17" t="str">
-        <f>A440</f>
-        <v>U+2205</v>
+      <c r="H440" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I440" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H440,3,4)))</f>
-        <v>∅</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="441" spans="1:11" ht="17" customHeight="1">
@@ -21126,7 +21157,7 @@
       </c>
       <c r="B441" s="5">
         <f>IF(ISNA(VLOOKUP(H441,$A$2:$C$1011,3,1)),C441,VLOOKUP(H441,$A$2:$C$1011,3,1))</f>
-        <v>668</v>
+        <v>663</v>
       </c>
       <c r="C441" s="1">
         <v>668</v>
@@ -21145,13 +21176,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A441,3,4)))</f>
         <v>∆</v>
       </c>
-      <c r="H441" s="17" t="str">
-        <f>A441</f>
-        <v>U+2206</v>
+      <c r="H441" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I441" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H441,3,4)))</f>
-        <v>∆</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="442" spans="1:11" ht="17" customHeight="1">
@@ -21160,7 +21190,7 @@
       </c>
       <c r="B442" s="5">
         <f>IF(ISNA(VLOOKUP(H442,$A$2:$C$1011,3,1)),C442,VLOOKUP(H442,$A$2:$C$1011,3,1))</f>
-        <v>669</v>
+        <v>663</v>
       </c>
       <c r="C442" s="1">
         <v>669</v>
@@ -21179,13 +21209,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A442,3,4)))</f>
         <v>∇</v>
       </c>
-      <c r="H442" s="17" t="str">
-        <f>A442</f>
-        <v>U+2207</v>
+      <c r="H442" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I442" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H442,3,4)))</f>
-        <v>∇</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="443" spans="1:11" ht="17" customHeight="1">
@@ -21194,7 +21223,7 @@
       </c>
       <c r="B443" s="5">
         <f>IF(ISNA(VLOOKUP(H443,$A$2:$C$1011,3,1)),C443,VLOOKUP(H443,$A$2:$C$1011,3,1))</f>
-        <v>670</v>
+        <v>663</v>
       </c>
       <c r="C443" s="1">
         <v>670</v>
@@ -21213,13 +21242,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A443,3,4)))</f>
         <v>∈</v>
       </c>
-      <c r="H443" s="17" t="str">
-        <f>A443</f>
-        <v>U+2208</v>
+      <c r="H443" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I443" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H443,3,4)))</f>
-        <v>∈</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="444" spans="1:11" ht="17" customHeight="1">
@@ -21228,7 +21256,7 @@
       </c>
       <c r="B444" s="5">
         <f>IF(ISNA(VLOOKUP(H444,$A$2:$C$1011,3,1)),C444,VLOOKUP(H444,$A$2:$C$1011,3,1))</f>
-        <v>671</v>
+        <v>663</v>
       </c>
       <c r="C444" s="1">
         <v>671</v>
@@ -21247,13 +21275,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A444,3,4)))</f>
         <v>∉</v>
       </c>
-      <c r="H444" s="17" t="str">
-        <f>A444</f>
-        <v>U+2209</v>
+      <c r="H444" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I444" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H444,3,4)))</f>
-        <v>∉</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="445" spans="1:11" ht="17" customHeight="1">
@@ -21262,7 +21289,7 @@
       </c>
       <c r="B445" s="5">
         <f>IF(ISNA(VLOOKUP(H445,$A$2:$C$1011,3,1)),C445,VLOOKUP(H445,$A$2:$C$1011,3,1))</f>
-        <v>672</v>
+        <v>663</v>
       </c>
       <c r="C445" s="1">
         <v>672</v>
@@ -21281,13 +21308,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A445,3,4)))</f>
         <v>∋</v>
       </c>
-      <c r="H445" s="17" t="str">
-        <f>A445</f>
-        <v>U+220b</v>
+      <c r="H445" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I445" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H445,3,4)))</f>
-        <v>∋</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="446" spans="1:11" ht="17" customHeight="1">
@@ -21296,7 +21322,7 @@
       </c>
       <c r="B446" s="5">
         <f>IF(ISNA(VLOOKUP(H446,$A$2:$C$1011,3,1)),C446,VLOOKUP(H446,$A$2:$C$1011,3,1))</f>
-        <v>673</v>
+        <v>663</v>
       </c>
       <c r="C446" s="1">
         <v>673</v>
@@ -21315,13 +21341,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A446,3,4)))</f>
         <v>∌</v>
       </c>
-      <c r="H446" s="17" t="str">
-        <f>A446</f>
-        <v>U+220c</v>
+      <c r="H446" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I446" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H446,3,4)))</f>
-        <v>∌</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="447" spans="1:11" ht="17" customHeight="1">
@@ -22023,7 +22048,7 @@
       </c>
       <c r="B468" s="5">
         <f>IF(ISNA(VLOOKUP(H468,$A$2:$C$1011,3,1)),C468,VLOOKUP(H468,$A$2:$C$1011,3,1))</f>
-        <v>674</v>
+        <v>663</v>
       </c>
       <c r="C468" s="1">
         <v>674</v>
@@ -22042,13 +22067,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A468,3,4)))</f>
         <v>∩</v>
       </c>
-      <c r="H468" s="17" t="str">
-        <f>A468</f>
-        <v>U+2229</v>
+      <c r="H468" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I468" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H468,3,4)))</f>
-        <v>∩</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="469" spans="1:9" ht="17" customHeight="1">
@@ -22057,7 +22081,7 @@
       </c>
       <c r="B469" s="5">
         <f>IF(ISNA(VLOOKUP(H469,$A$2:$C$1011,3,1)),C469,VLOOKUP(H469,$A$2:$C$1011,3,1))</f>
-        <v>675</v>
+        <v>663</v>
       </c>
       <c r="C469" s="1">
         <v>675</v>
@@ -22076,13 +22100,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A469,3,4)))</f>
         <v>∪</v>
       </c>
-      <c r="H469" s="17" t="str">
-        <f>A469</f>
-        <v>U+222a</v>
+      <c r="H469" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I469" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H469,3,4)))</f>
-        <v>∪</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="470" spans="1:9" ht="17" customHeight="1">
@@ -22685,7 +22708,7 @@
       </c>
       <c r="B488" s="5">
         <f>IF(ISNA(VLOOKUP(H488,$A$2:$C$1011,3,1)),C488,VLOOKUP(H488,$A$2:$C$1011,3,1))</f>
-        <v>676</v>
+        <v>663</v>
       </c>
       <c r="C488" s="1">
         <v>676</v>
@@ -22704,13 +22727,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A488,3,4)))</f>
         <v>⊂</v>
       </c>
-      <c r="H488" s="17" t="str">
-        <f>A488</f>
-        <v>U+2282</v>
+      <c r="H488" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I488" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H488,3,4)))</f>
-        <v>⊂</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="489" spans="1:9" ht="17" customHeight="1">
@@ -22719,7 +22741,7 @@
       </c>
       <c r="B489" s="5">
         <f>IF(ISNA(VLOOKUP(H489,$A$2:$C$1011,3,1)),C489,VLOOKUP(H489,$A$2:$C$1011,3,1))</f>
-        <v>677</v>
+        <v>663</v>
       </c>
       <c r="C489" s="1">
         <v>677</v>
@@ -22738,13 +22760,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A489,3,4)))</f>
         <v>⊄</v>
       </c>
-      <c r="H489" s="17" t="str">
-        <f>A489</f>
-        <v>U+2284</v>
+      <c r="H489" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I489" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H489,3,4)))</f>
-        <v>⊄</v>
+        <v>Ɐ</v>
       </c>
     </row>
     <row r="490" spans="1:9" ht="17" customHeight="1">
@@ -23182,7 +23203,7 @@
       </c>
       <c r="B503" s="5">
         <f>IF(ISNA(VLOOKUP(H503,$A$2:$C$1011,3,1)),C503,VLOOKUP(H503,$A$2:$C$1011,3,1))</f>
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="C503" s="1">
         <v>643</v>
@@ -23201,13 +23222,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A503,3,4)))</f>
         <v>⌚</v>
       </c>
-      <c r="H503" s="17" t="str">
-        <f>A503</f>
-        <v>U+231a</v>
+      <c r="H503" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I503" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H503,3,4)))</f>
-        <v>⌚</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="504" spans="1:9" ht="17" customHeight="1">
@@ -23216,7 +23236,7 @@
       </c>
       <c r="B504" s="5">
         <f>IF(ISNA(VLOOKUP(H504,$A$2:$C$1011,3,1)),C504,VLOOKUP(H504,$A$2:$C$1011,3,1))</f>
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="C504" s="1">
         <v>641</v>
@@ -23235,13 +23255,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A504,3,4)))</f>
         <v>⌛</v>
       </c>
-      <c r="H504" s="17" t="str">
-        <f>A504</f>
-        <v>U+231b</v>
+      <c r="H504" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I504" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H504,3,4)))</f>
-        <v>⌛</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="505" spans="1:9" ht="17" customHeight="1">
@@ -23302,9 +23321,8 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A506,3,4)))</f>
         <v>⎙</v>
       </c>
-      <c r="H506" s="17" t="str">
-        <f>A506</f>
-        <v>U+2399</v>
+      <c r="H506" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I506" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H506,3,4)))</f>
@@ -23581,7 +23599,7 @@
       </c>
       <c r="B515" s="5">
         <f>IF(ISNA(VLOOKUP(H515,$A$2:$C$1011,3,1)),C515,VLOOKUP(H515,$A$2:$C$1011,3,1))</f>
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="C515" s="1">
         <v>644</v>
@@ -23600,13 +23618,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A515,3,4)))</f>
         <v>⏱</v>
       </c>
-      <c r="H515" s="17" t="str">
-        <f>A515</f>
-        <v>U+23f1</v>
+      <c r="H515" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I515" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H515,3,4)))</f>
-        <v>⏱</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="516" spans="1:9" ht="17" customHeight="1">
@@ -23615,7 +23632,7 @@
       </c>
       <c r="B516" s="5">
         <f>IF(ISNA(VLOOKUP(H516,$A$2:$C$1011,3,1)),C516,VLOOKUP(H516,$A$2:$C$1011,3,1))</f>
-        <v>651</v>
+        <v>640</v>
       </c>
       <c r="C516" s="1">
         <v>651</v>
@@ -23634,13 +23651,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A516,3,4)))</f>
         <v>⏻</v>
       </c>
-      <c r="H516" s="17" t="str">
-        <f>A516</f>
-        <v>U+23fb</v>
+      <c r="H516" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I516" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H516,3,4)))</f>
-        <v>⏻</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="517" spans="1:9" ht="17" customHeight="1">
@@ -23668,9 +23684,8 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A517,3,4)))</f>
         <v>␡</v>
       </c>
-      <c r="H517" s="17" t="str">
-        <f>A517</f>
-        <v>U+2421</v>
+      <c r="H517" s="21" t="s">
+        <v>1525</v>
       </c>
       <c r="I517" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H517,3,4)))</f>
@@ -23683,7 +23698,7 @@
       </c>
       <c r="B518" s="5">
         <f>IF(ISNA(VLOOKUP(H518,$A$2:$C$1011,3,1)),C518,VLOOKUP(H518,$A$2:$C$1011,3,1))</f>
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="C518" s="1">
         <v>679</v>
@@ -23702,13 +23717,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A518,3,4)))</f>
         <v>␢</v>
       </c>
-      <c r="H518" s="17" t="str">
-        <f>A518</f>
-        <v>U+2422</v>
+      <c r="H518" s="21" t="s">
+        <v>1525</v>
       </c>
       <c r="I518" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H518,3,4)))</f>
-        <v>␢</v>
+        <v>␡</v>
       </c>
     </row>
     <row r="519" spans="1:9" ht="17" customHeight="1">
@@ -23750,7 +23764,7 @@
       </c>
       <c r="B520" s="5">
         <f>IF(ISNA(VLOOKUP(H520,$A$2:$C$1011,3,1)),C520,VLOOKUP(H520,$A$2:$C$1011,3,1))</f>
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="C520" s="1">
         <v>680</v>
@@ -23769,13 +23783,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A520,3,4)))</f>
         <v>␥</v>
       </c>
-      <c r="H520" s="17" t="str">
-        <f>A520</f>
-        <v>U+2425</v>
+      <c r="H520" s="21" t="s">
+        <v>1525</v>
       </c>
       <c r="I520" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H520,3,4)))</f>
-        <v>␥</v>
+        <v>␡</v>
       </c>
     </row>
     <row r="521" spans="1:9" ht="17" customHeight="1">
@@ -23784,7 +23797,7 @@
       </c>
       <c r="B521" s="5">
         <f>IF(ISNA(VLOOKUP(H521,$A$2:$C$1011,3,1)),C521,VLOOKUP(H521,$A$2:$C$1011,3,1))</f>
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C521" s="1">
         <v>681</v>
@@ -23803,13 +23816,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A521,3,4)))</f>
         <v>␦</v>
       </c>
-      <c r="H521" s="17" t="str">
-        <f>A521</f>
-        <v>U+2426</v>
+      <c r="H521" s="21" t="s">
+        <v>1525</v>
       </c>
       <c r="I521" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H521,3,4)))</f>
-        <v>␦</v>
+        <v>␡</v>
       </c>
     </row>
     <row r="522" spans="1:9" ht="17" customHeight="1">
@@ -23917,7 +23929,7 @@
       </c>
       <c r="B525" s="5">
         <f>IF(ISNA(VLOOKUP(H525,$A$2:$C$1011,3,1)),C525,VLOOKUP(H525,$A$2:$C$1011,3,1))</f>
-        <v>645</v>
+        <v>640</v>
       </c>
       <c r="C525" s="1">
         <v>645</v>
@@ -23936,13 +23948,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A525,3,4)))</f>
         <v>␪</v>
       </c>
-      <c r="H525" s="17" t="str">
-        <f>A525</f>
-        <v>U+242a</v>
+      <c r="H525" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I525" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H525,3,4)))</f>
-        <v>␪</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="526" spans="1:9" ht="17" customHeight="1">
@@ -23984,7 +23995,7 @@
       </c>
       <c r="B527" s="5">
         <f>IF(ISNA(VLOOKUP(H527,$A$2:$C$1011,3,1)),C527,VLOOKUP(H527,$A$2:$C$1011,3,1))</f>
-        <v>647</v>
+        <v>640</v>
       </c>
       <c r="C527" s="1">
         <v>647</v>
@@ -24003,13 +24014,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A527,3,4)))</f>
         <v>␬</v>
       </c>
-      <c r="H527" s="17" t="str">
-        <f>A527</f>
-        <v>U+242c</v>
+      <c r="H527" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I527" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H527,3,4)))</f>
-        <v>␬</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="528" spans="1:9" ht="17" customHeight="1">
@@ -24037,9 +24047,8 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A528,3,4)))</f>
         <v>␭</v>
       </c>
-      <c r="H528" s="17" t="str">
-        <f>A528</f>
-        <v>U+242d</v>
+      <c r="H528" s="19" t="s">
+        <v>1551</v>
       </c>
       <c r="I528" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H528,3,4)))</f>
@@ -24052,7 +24061,7 @@
       </c>
       <c r="B529" s="5">
         <f>IF(ISNA(VLOOKUP(H529,$A$2:$C$1011,3,1)),C529,VLOOKUP(H529,$A$2:$C$1011,3,1))</f>
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C529" s="1">
         <v>662</v>
@@ -24071,13 +24080,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A529,3,4)))</f>
         <v>␮</v>
       </c>
-      <c r="H529" s="17" t="str">
-        <f>A529</f>
-        <v>U+242e</v>
+      <c r="H529" s="19" t="s">
+        <v>1551</v>
       </c>
       <c r="I529" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H529,3,4)))</f>
-        <v>␮</v>
+        <v>␭</v>
       </c>
     </row>
     <row r="530" spans="1:9" ht="17" customHeight="1">
@@ -24086,7 +24094,7 @@
       </c>
       <c r="B530" s="5">
         <f>IF(ISNA(VLOOKUP(H530,$A$2:$C$1011,3,1)),C530,VLOOKUP(H530,$A$2:$C$1011,3,1))</f>
-        <v>648</v>
+        <v>640</v>
       </c>
       <c r="C530" s="1">
         <v>648</v>
@@ -24105,13 +24113,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A530,3,4)))</f>
         <v>␯</v>
       </c>
-      <c r="H530" s="17" t="str">
-        <f>A530</f>
-        <v>U+242f</v>
+      <c r="H530" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I530" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H530,3,4)))</f>
-        <v>␯</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="531" spans="1:9" ht="17" customHeight="1">
@@ -24252,7 +24259,7 @@
       </c>
       <c r="B535" s="5">
         <f>IF(ISNA(VLOOKUP(H535,$A$2:$C$1011,3,1)),C535,VLOOKUP(H535,$A$2:$C$1011,3,1))</f>
-        <v>649</v>
+        <v>640</v>
       </c>
       <c r="C535" s="1">
         <v>649</v>
@@ -24271,13 +24278,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A535,3,4)))</f>
         <v>␴</v>
       </c>
-      <c r="H535" s="17" t="str">
-        <f>A535</f>
-        <v>U+2434</v>
+      <c r="H535" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I535" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H535,3,4)))</f>
-        <v>␴</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="536" spans="1:9" ht="17" customHeight="1">
@@ -24286,7 +24292,7 @@
       </c>
       <c r="B536" s="5">
         <f>IF(ISNA(VLOOKUP(H536,$A$2:$C$1011,3,1)),C536,VLOOKUP(H536,$A$2:$C$1011,3,1))</f>
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="C536" s="1">
         <v>646</v>
@@ -24305,13 +24311,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A536,3,4)))</f>
         <v>␵</v>
       </c>
-      <c r="H536" s="17" t="str">
-        <f>A536</f>
-        <v>U+2435</v>
+      <c r="H536" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I536" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H536,3,4)))</f>
-        <v>␵</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="537" spans="1:9" ht="17" customHeight="1">
@@ -28349,7 +28354,7 @@
       </c>
       <c r="B659" s="5">
         <f>IF(ISNA(VLOOKUP(H659,$A$2:$C$1011,3,1)),C659,VLOOKUP(H659,$A$2:$C$1011,3,1))</f>
-        <v>652</v>
+        <v>640</v>
       </c>
       <c r="C659" s="1">
         <v>652</v>
@@ -28368,13 +28373,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A659,3,4)))</f>
         <v>▢</v>
       </c>
-      <c r="H659" s="17" t="str">
-        <f>A659</f>
-        <v>U+25a2</v>
+      <c r="H659" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I659" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H659,3,4)))</f>
-        <v>▢</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="660" spans="1:9" ht="17" customHeight="1">
@@ -28383,7 +28387,7 @@
       </c>
       <c r="B660" s="5">
         <f>IF(ISNA(VLOOKUP(H660,$A$2:$C$1011,3,1)),C660,VLOOKUP(H660,$A$2:$C$1011,3,1))</f>
-        <v>653</v>
+        <v>640</v>
       </c>
       <c r="C660" s="1">
         <v>653</v>
@@ -28402,13 +28406,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A660,3,4)))</f>
         <v>▦</v>
       </c>
-      <c r="H660" s="17" t="str">
-        <f>A660</f>
-        <v>U+25a6</v>
+      <c r="H660" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I660" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H660,3,4)))</f>
-        <v>▦</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="661" spans="1:9" ht="17" customHeight="1">
@@ -28417,7 +28420,7 @@
       </c>
       <c r="B661" s="5">
         <f>IF(ISNA(VLOOKUP(H661,$A$2:$C$1011,3,1)),C661,VLOOKUP(H661,$A$2:$C$1011,3,1))</f>
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="C661" s="1">
         <v>658</v>
@@ -28436,13 +28439,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A661,3,4)))</f>
         <v>◇</v>
       </c>
-      <c r="H661" s="17" t="str">
-        <f>A661</f>
-        <v>U+25c7</v>
+      <c r="H661" s="18" t="s">
+        <v>2009</v>
       </c>
       <c r="I661" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H661,3,4)))</f>
-        <v>◇</v>
+        <v>◯</v>
       </c>
     </row>
     <row r="662" spans="1:9" ht="17" customHeight="1">
@@ -28451,7 +28453,7 @@
       </c>
       <c r="B662" s="5">
         <f>IF(ISNA(VLOOKUP(H662,$A$2:$C$1011,3,1)),C662,VLOOKUP(H662,$A$2:$C$1011,3,1))</f>
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="C662" s="1">
         <v>659</v>
@@ -28470,13 +28472,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A662,3,4)))</f>
         <v>◈</v>
       </c>
-      <c r="H662" s="17" t="str">
-        <f>A662</f>
-        <v>U+25c8</v>
+      <c r="H662" s="18" t="s">
+        <v>2009</v>
       </c>
       <c r="I662" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H662,3,4)))</f>
-        <v>◈</v>
+        <v>◯</v>
       </c>
     </row>
     <row r="663" spans="1:9" ht="17" customHeight="1">
@@ -28504,9 +28505,8 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A663,3,4)))</f>
         <v>◯</v>
       </c>
-      <c r="H663" s="17" t="str">
-        <f>A663</f>
-        <v>U+25ef</v>
+      <c r="H663" s="18" t="s">
+        <v>2009</v>
       </c>
       <c r="I663" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H663,3,4)))</f>
@@ -28519,7 +28519,7 @@
       </c>
       <c r="B664" s="5">
         <f>IF(ISNA(VLOOKUP(H664,$A$2:$C$1011,3,1)),C664,VLOOKUP(H664,$A$2:$C$1011,3,1))</f>
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="C664" s="1">
         <v>654</v>
@@ -28538,13 +28538,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A664,3,4)))</f>
         <v>☐</v>
       </c>
-      <c r="H664" s="17" t="str">
-        <f>A664</f>
-        <v>U+2610</v>
+      <c r="H664" s="18" t="s">
+        <v>2009</v>
       </c>
       <c r="I664" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H664,3,4)))</f>
-        <v>☐</v>
+        <v>◯</v>
       </c>
     </row>
     <row r="665" spans="1:9" ht="17" customHeight="1">
@@ -28553,7 +28552,7 @@
       </c>
       <c r="B665" s="5">
         <f>IF(ISNA(VLOOKUP(H665,$A$2:$C$1011,3,1)),C665,VLOOKUP(H665,$A$2:$C$1011,3,1))</f>
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C665" s="1">
         <v>655</v>
@@ -28572,13 +28571,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A665,3,4)))</f>
         <v>☒</v>
       </c>
-      <c r="H665" s="17" t="str">
-        <f>A665</f>
-        <v>U+2612</v>
+      <c r="H665" s="18" t="s">
+        <v>2009</v>
       </c>
       <c r="I665" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H665,3,4)))</f>
-        <v>☒</v>
+        <v>◯</v>
       </c>
     </row>
     <row r="666" spans="1:9" ht="17" customHeight="1">
@@ -28587,7 +28585,7 @@
       </c>
       <c r="B666" s="5">
         <f>IF(ISNA(VLOOKUP(H666,$A$2:$C$1011,3,1)),C666,VLOOKUP(H666,$A$2:$C$1011,3,1))</f>
-        <v>650</v>
+        <v>640</v>
       </c>
       <c r="C666" s="1">
         <v>650</v>
@@ -28606,13 +28604,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A666,3,4)))</f>
         <v>♺</v>
       </c>
-      <c r="H666" s="17" t="str">
-        <f>A666</f>
-        <v>U+267A</v>
+      <c r="H666" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I666" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H666,3,4)))</f>
-        <v>♺</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="667" spans="1:9" ht="17" customHeight="1">
@@ -28786,7 +28783,7 @@
       </c>
       <c r="B672" s="5">
         <f>IF(ISNA(VLOOKUP(H672,$A$2:$C$1011,3,1)),C672,VLOOKUP(H672,$A$2:$C$1011,3,1))</f>
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="C672" s="1">
         <v>657</v>
@@ -28805,13 +28802,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A672,3,4)))</f>
         <v>⦿</v>
       </c>
-      <c r="H672" s="17" t="str">
-        <f>A672</f>
-        <v>U+29bf</v>
+      <c r="H672" s="18" t="s">
+        <v>2009</v>
       </c>
       <c r="I672" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H672,3,4)))</f>
-        <v>⦿</v>
+        <v>◯</v>
       </c>
     </row>
     <row r="673" spans="1:11" ht="17" customHeight="1">
@@ -28820,7 +28816,7 @@
       </c>
       <c r="B673" s="5">
         <f>IF(ISNA(VLOOKUP(H673,$A$2:$C$1011,3,1)),C673,VLOOKUP(H673,$A$2:$C$1011,3,1))</f>
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="C673" s="1">
         <v>642</v>
@@ -28839,13 +28835,12 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A673,3,4)))</f>
         <v>⧖</v>
       </c>
-      <c r="H673" s="17" t="str">
-        <f>A673</f>
-        <v>U+29d6</v>
+      <c r="H673" s="17" t="s">
+        <v>1486</v>
       </c>
       <c r="I673" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H673,3,4)))</f>
-        <v>⧖</v>
+        <v>⎙</v>
       </c>
     </row>
     <row r="674" spans="1:11" ht="17" customHeight="1">
@@ -29170,9 +29165,8 @@
         <f>_xlfn.UNICHAR(HEX2DEC(MID(A683,3,4)))</f>
         <v>Ɐ</v>
       </c>
-      <c r="H683" s="17" t="str">
-        <f>A683</f>
-        <v>U+2c6f</v>
+      <c r="H683" s="20" t="s">
+        <v>1289</v>
       </c>
       <c r="I683" s="6" t="str">
         <f>_xlfn.UNICHAR(HEX2DEC(MID(H683,3,4)))</f>
@@ -29267,8 +29261,8 @@
       <c r="K714" s="2"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I715">
-    <sortCondition ref="A2:A715"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K714">
+    <sortCondition ref="A2:A714"/>
   </sortState>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>